<commit_message>
데이터 수정 - Target Value
</commit_message>
<xml_diff>
--- a/template/1-1. 전사인력산정용_R&A.xlsx
+++ b/template/1-1. 전사인력산정용_R&A.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://insightgroup2006.sharepoint.com/sites/msteams_0b54cd/Shared Documents/일반/02. 프로젝트 진행/04. Data/0. Master Template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hanskim/Projects/Hwaseung/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{80F058D4-9BDF-435B-B863-71C145C8F2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73D89A77-F8B2-43F7-9448-4AECDB46CB40}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FFE629-87B7-E249-B1F3-7EFFE6812967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6BEFEA37-F532-4AD1-8EF6-045DD3318223}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="29560" windowHeight="11500" xr2:uid="{6BEFEA37-F532-4AD1-8EF6-045DD3318223}"/>
   </bookViews>
   <sheets>
     <sheet name="master" sheetId="1" r:id="rId1"/>
@@ -148,7 +148,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,27 +556,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09995889-7D11-483A-B8E4-8DCF236E8E82}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.4140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.08203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.08203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.08203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15" style="1" customWidth="1"/>
     <col min="16" max="16" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,7 +626,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -676,7 +676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16">
       <c r="A3" s="1">
         <v>2021</v>
       </c>
@@ -726,7 +726,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16">
       <c r="A4" s="1">
         <v>2022</v>
       </c>
@@ -776,7 +776,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16">
       <c r="A5" s="1">
         <v>2023</v>
       </c>
@@ -826,7 +826,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16">
       <c r="A6" s="1">
         <v>2024</v>
       </c>
@@ -876,7 +876,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16">
       <c r="A7" s="1">
         <v>2025</v>
       </c>
@@ -919,8 +919,8 @@
       <c r="N7" s="1">
         <v>-1.7167381974248927E-2</v>
       </c>
-      <c r="P7" s="1">
-        <v>256</v>
+      <c r="O7" s="1">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -930,12 +930,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="72a48f7e-7092-4e54-b227-c271416f5cc4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="97fdf058-3532-4042-931f-ee11ab7234aa" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1134,20 +1136,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="72a48f7e-7092-4e54-b227-c271416f5cc4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="97fdf058-3532-4042-931f-ee11ab7234aa" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29422BF8-1DB7-4D92-B788-79F3D7AF4E7A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3F1CA8F-A330-49D3-A613-D931FC9DDBA3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="72a48f7e-7092-4e54-b227-c271416f5cc4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="97fdf058-3532-4042-931f-ee11ab7234aa"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1172,18 +1181,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3F1CA8F-A330-49D3-A613-D931FC9DDBA3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29422BF8-1DB7-4D92-B788-79F3D7AF4E7A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="72a48f7e-7092-4e54-b227-c271416f5cc4"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="97fdf058-3532-4042-931f-ee11ab7234aa"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>